<commit_message>
updated script to use root level project directory
</commit_message>
<xml_diff>
--- a/mobile/scripts/ingestion.xlsx
+++ b/mobile/scripts/ingestion.xlsx
@@ -1,6 +1,6 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ns2="http://schemas.libreoffice.org/" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <fileVersion appName="Calc"/>
   <workbookPr backupFile="false" showObjects="all" date1904="false"/>
   <workbookProtection/>
@@ -10,14 +10,12 @@
   <sheets>
     <sheet name="ActivityFacilities" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Assets" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="BOMValues" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Helpers" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="_DropdownValues" sheetId="5" state="hidden" r:id="rId7"/>
+    <sheet name="_DropdownValues" sheetId="3" state="hidden" r:id="rId7"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
-    <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
-      <loext:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
+    <ext uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
+      <ns2:extCalcPr stringRefSyntax="CalcA1ExcelA1"/>
     </ext>
   </extLst>
 </workbook>
@@ -810,7 +808,7 @@
   </headerFooter>
   <dataValidations count="1">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B1000">
-      <formula1>_DropdownValues!$A$2:$A$4</formula1>
+      <formula1>_DropdownValues!$A$2:$A$5</formula1>
     </dataValidation>
   </dataValidations>
 </worksheet>
@@ -1393,37 +1391,52 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
-  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <dimension ref="A1:A5"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="2" width="16.34"/>
+    <col min="1" max="1" width="16" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>110</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="2" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A3" s="2" t="s">
-        <v>22</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="2" t="s">
-        <v>28</v>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>AssetTypes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>inverter</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>battery</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>panel</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>RMS</t>
+        </is>
       </c>
     </row>
   </sheetData>
+  <sheetFormatPr defaultColWidth="8.6875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.747916666666667" right="0.747916666666667" top="0.984027777777778" bottom="0.984027777777778" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>

</xml_diff>